<commit_message>
update data gen and configs
</commit_message>
<xml_diff>
--- a/data_generation/andes_cases/ieee39_full.xlsx
+++ b/data_generation/andes_cases/ieee39_full.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cloud9/Desktop/ETH Project/Working folder/03_Code/vis-ml/data_generation/andes_cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D57A4C-D084-E841-886D-D02A3310D003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FDC897C-A978-F342-A83D-53EB8AFC8B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="9120" windowWidth="30240" windowHeight="8820" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,9 @@
     <sheet name="GENROU" sheetId="8" r:id="rId8"/>
     <sheet name="COI" sheetId="15" r:id="rId9"/>
     <sheet name="TGOV1N" sheetId="9" r:id="rId10"/>
-    <sheet name="BusFreq" sheetId="12" r:id="rId11"/>
+    <sheet name="IEEEST" sheetId="18" r:id="rId11"/>
+    <sheet name="IEEEX1" sheetId="17" r:id="rId12"/>
+    <sheet name="BusFreq" sheetId="12" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="263">
   <si>
     <t>idx</t>
   </si>
@@ -674,6 +676,162 @@
   </si>
   <si>
     <t>COI_1</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>TA</t>
+  </si>
+  <si>
+    <t>TC</t>
+  </si>
+  <si>
+    <t>TB</t>
+  </si>
+  <si>
+    <t>TE</t>
+  </si>
+  <si>
+    <t>TF1</t>
+  </si>
+  <si>
+    <t>KF1</t>
+  </si>
+  <si>
+    <t>KA</t>
+  </si>
+  <si>
+    <t>KE</t>
+  </si>
+  <si>
+    <t>VRMAX</t>
+  </si>
+  <si>
+    <t>VRMIN</t>
+  </si>
+  <si>
+    <t>E1</t>
+  </si>
+  <si>
+    <t>SE1</t>
+  </si>
+  <si>
+    <t>E2</t>
+  </si>
+  <si>
+    <t>SE2</t>
+  </si>
+  <si>
+    <t>IEEEX1_1</t>
+  </si>
+  <si>
+    <t>IEEEX1_2</t>
+  </si>
+  <si>
+    <t>IEEEX1_3</t>
+  </si>
+  <si>
+    <t>IEEEX1_4</t>
+  </si>
+  <si>
+    <t>IEEEX1_5</t>
+  </si>
+  <si>
+    <t>IEEEX1_6</t>
+  </si>
+  <si>
+    <t>IEEEX1_7</t>
+  </si>
+  <si>
+    <t>IEEEX1_8</t>
+  </si>
+  <si>
+    <t>IEEEX1_9</t>
+  </si>
+  <si>
+    <t>IEEEX1_10</t>
+  </si>
+  <si>
+    <t>avr</t>
+  </si>
+  <si>
+    <t>MODE</t>
+  </si>
+  <si>
+    <t>busf</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t>T6</t>
+  </si>
+  <si>
+    <t>KS</t>
+  </si>
+  <si>
+    <t>LSMAX</t>
+  </si>
+  <si>
+    <t>LSMIN</t>
+  </si>
+  <si>
+    <t>VCU</t>
+  </si>
+  <si>
+    <t>VCL</t>
+  </si>
+  <si>
+    <t>IEEEST_1</t>
+  </si>
+  <si>
+    <t>IEEEST_2</t>
+  </si>
+  <si>
+    <t>IEEEST_3</t>
+  </si>
+  <si>
+    <t>IEEEST_4</t>
+  </si>
+  <si>
+    <t>IEEEST_5</t>
+  </si>
+  <si>
+    <t>IEEEST_6</t>
+  </si>
+  <si>
+    <t>IEEEST_7</t>
+  </si>
+  <si>
+    <t>IEEEST_8</t>
+  </si>
+  <si>
+    <t>IEEEST_9</t>
+  </si>
+  <si>
+    <t>IEEEST_10</t>
   </si>
 </sst>
 </file>
@@ -2911,7 +3069,7 @@
         <v>1.01</v>
       </c>
       <c r="J2">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>0.05</v>
@@ -2952,7 +3110,7 @@
         <v>1.05</v>
       </c>
       <c r="J3">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K3">
         <v>0.05</v>
@@ -2993,7 +3151,7 @@
         <v>1.05</v>
       </c>
       <c r="J4">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>0.05</v>
@@ -3034,7 +3192,7 @@
         <v>1.05</v>
       </c>
       <c r="J5">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K5">
         <v>0.05</v>
@@ -3075,7 +3233,7 @@
         <v>1.05</v>
       </c>
       <c r="J6">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <v>0.05</v>
@@ -3116,7 +3274,7 @@
         <v>1.05</v>
       </c>
       <c r="J7">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K7">
         <v>0.05</v>
@@ -3157,7 +3315,7 @@
         <v>1.05</v>
       </c>
       <c r="J8">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <v>0.05</v>
@@ -3198,7 +3356,7 @@
         <v>1.05</v>
       </c>
       <c r="J9">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K9">
         <v>0.05</v>
@@ -3239,7 +3397,7 @@
         <v>1.05</v>
       </c>
       <c r="J10">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K10">
         <v>0.05</v>
@@ -3280,7 +3438,7 @@
         <v>1.05</v>
       </c>
       <c r="J11">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K11">
         <v>0.05</v>
@@ -3301,6 +3459,1525 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AAAFFDB-3D26-1446-A9BB-24A725154BAE}">
+  <dimension ref="A1:Y11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
+        <v>198</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0.75</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
+      </c>
+      <c r="T2">
+        <v>4.2</v>
+      </c>
+      <c r="U2">
+        <v>-2</v>
+      </c>
+      <c r="V2">
+        <v>0.1</v>
+      </c>
+      <c r="W2">
+        <v>-0.1</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>254</v>
+      </c>
+      <c r="E3" t="s">
+        <v>227</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="H3" t="s">
+        <v>199</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0.75</v>
+      </c>
+      <c r="S3">
+        <v>1</v>
+      </c>
+      <c r="T3">
+        <v>4.2</v>
+      </c>
+      <c r="U3">
+        <v>-2</v>
+      </c>
+      <c r="V3">
+        <v>0.1</v>
+      </c>
+      <c r="W3">
+        <v>-0.1</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>255</v>
+      </c>
+      <c r="E4" t="s">
+        <v>228</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="H4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0.75</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
+      </c>
+      <c r="T4">
+        <v>4.2</v>
+      </c>
+      <c r="U4">
+        <v>-2</v>
+      </c>
+      <c r="V4">
+        <v>0.1</v>
+      </c>
+      <c r="W4">
+        <v>-0.1</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>256</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>256</v>
+      </c>
+      <c r="E5" t="s">
+        <v>229</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="H5" t="s">
+        <v>201</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0.75</v>
+      </c>
+      <c r="S5">
+        <v>1</v>
+      </c>
+      <c r="T5">
+        <v>4.2</v>
+      </c>
+      <c r="U5">
+        <v>-2</v>
+      </c>
+      <c r="V5">
+        <v>0.1</v>
+      </c>
+      <c r="W5">
+        <v>-0.1</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>257</v>
+      </c>
+      <c r="E6" t="s">
+        <v>230</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="H6" t="s">
+        <v>202</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0.75</v>
+      </c>
+      <c r="S6">
+        <v>1</v>
+      </c>
+      <c r="T6">
+        <v>4.2</v>
+      </c>
+      <c r="U6">
+        <v>-2</v>
+      </c>
+      <c r="V6">
+        <v>0.1</v>
+      </c>
+      <c r="W6">
+        <v>-0.1</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>258</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>258</v>
+      </c>
+      <c r="E7" t="s">
+        <v>231</v>
+      </c>
+      <c r="F7">
+        <v>3</v>
+      </c>
+      <c r="H7" t="s">
+        <v>203</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0.75</v>
+      </c>
+      <c r="S7">
+        <v>1</v>
+      </c>
+      <c r="T7">
+        <v>4.2</v>
+      </c>
+      <c r="U7">
+        <v>-2</v>
+      </c>
+      <c r="V7">
+        <v>0.1</v>
+      </c>
+      <c r="W7">
+        <v>-0.1</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>259</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>259</v>
+      </c>
+      <c r="E8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
+      </c>
+      <c r="H8" t="s">
+        <v>204</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>0.75</v>
+      </c>
+      <c r="S8">
+        <v>1</v>
+      </c>
+      <c r="T8">
+        <v>4.2</v>
+      </c>
+      <c r="U8">
+        <v>-2</v>
+      </c>
+      <c r="V8">
+        <v>0.1</v>
+      </c>
+      <c r="W8">
+        <v>-0.1</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>260</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>260</v>
+      </c>
+      <c r="E9" t="s">
+        <v>233</v>
+      </c>
+      <c r="F9">
+        <v>3</v>
+      </c>
+      <c r="H9" t="s">
+        <v>205</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>0.75</v>
+      </c>
+      <c r="S9">
+        <v>1</v>
+      </c>
+      <c r="T9">
+        <v>4.2</v>
+      </c>
+      <c r="U9">
+        <v>-2</v>
+      </c>
+      <c r="V9">
+        <v>0.1</v>
+      </c>
+      <c r="W9">
+        <v>-0.1</v>
+      </c>
+      <c r="X9">
+        <v>0</v>
+      </c>
+      <c r="Y9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>261</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>261</v>
+      </c>
+      <c r="E10" t="s">
+        <v>234</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="H10" t="s">
+        <v>206</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0.75</v>
+      </c>
+      <c r="S10">
+        <v>1</v>
+      </c>
+      <c r="T10">
+        <v>4.2</v>
+      </c>
+      <c r="U10">
+        <v>-2</v>
+      </c>
+      <c r="V10">
+        <v>0.1</v>
+      </c>
+      <c r="W10">
+        <v>-0.1</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>262</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>262</v>
+      </c>
+      <c r="E11" t="s">
+        <v>235</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="H11" t="s">
+        <v>207</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>0.75</v>
+      </c>
+      <c r="S11">
+        <v>1</v>
+      </c>
+      <c r="T11">
+        <v>4.2</v>
+      </c>
+      <c r="U11">
+        <v>-2</v>
+      </c>
+      <c r="V11">
+        <v>0.1</v>
+      </c>
+      <c r="W11">
+        <v>-0.1</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EFF0782-6D4A-9F4C-AAF0-36C9E1F16EF9}">
+  <dimension ref="A1:T11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E2" t="s">
+        <v>168</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0.06</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0.25</v>
+      </c>
+      <c r="K2">
+        <v>1.3</v>
+      </c>
+      <c r="L2">
+        <v>0.23</v>
+      </c>
+      <c r="M2">
+        <v>10.1</v>
+      </c>
+      <c r="N2">
+        <v>-0.05</v>
+      </c>
+      <c r="O2">
+        <v>8</v>
+      </c>
+      <c r="P2">
+        <v>-8</v>
+      </c>
+      <c r="Q2">
+        <v>1.7</v>
+      </c>
+      <c r="R2">
+        <v>0.5</v>
+      </c>
+      <c r="S2">
+        <v>3</v>
+      </c>
+      <c r="T2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>227</v>
+      </c>
+      <c r="E3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0.05</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0.41</v>
+      </c>
+      <c r="K3">
+        <v>1.3</v>
+      </c>
+      <c r="L3">
+        <v>0.23</v>
+      </c>
+      <c r="M3">
+        <v>10.1</v>
+      </c>
+      <c r="N3">
+        <v>-0.05</v>
+      </c>
+      <c r="O3">
+        <v>5.2</v>
+      </c>
+      <c r="P3">
+        <v>-5</v>
+      </c>
+      <c r="Q3">
+        <v>3</v>
+      </c>
+      <c r="R3">
+        <v>0.66</v>
+      </c>
+      <c r="S3">
+        <v>4</v>
+      </c>
+      <c r="T3">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0.06</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0.5</v>
+      </c>
+      <c r="K4">
+        <v>1.3</v>
+      </c>
+      <c r="L4">
+        <v>0.23</v>
+      </c>
+      <c r="M4">
+        <v>10.1</v>
+      </c>
+      <c r="N4">
+        <v>-0.02</v>
+      </c>
+      <c r="O4">
+        <v>5</v>
+      </c>
+      <c r="P4">
+        <v>-5</v>
+      </c>
+      <c r="Q4">
+        <v>3</v>
+      </c>
+      <c r="R4">
+        <v>0.13</v>
+      </c>
+      <c r="S4">
+        <v>4</v>
+      </c>
+      <c r="T4">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>229</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>229</v>
+      </c>
+      <c r="E5" t="s">
+        <v>171</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0.06</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0.5</v>
+      </c>
+      <c r="K5">
+        <v>1.3</v>
+      </c>
+      <c r="L5">
+        <v>0.23</v>
+      </c>
+      <c r="M5">
+        <v>10.1</v>
+      </c>
+      <c r="N5">
+        <v>-0.05</v>
+      </c>
+      <c r="O5">
+        <v>5</v>
+      </c>
+      <c r="P5">
+        <v>-5</v>
+      </c>
+      <c r="Q5">
+        <v>3</v>
+      </c>
+      <c r="R5">
+        <v>0.08</v>
+      </c>
+      <c r="S5">
+        <v>4</v>
+      </c>
+      <c r="T5">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>230</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>230</v>
+      </c>
+      <c r="E6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0.02</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0.78500000000000003</v>
+      </c>
+      <c r="K6">
+        <v>1.3</v>
+      </c>
+      <c r="L6">
+        <v>0.23</v>
+      </c>
+      <c r="M6">
+        <v>40</v>
+      </c>
+      <c r="N6">
+        <v>-0.04</v>
+      </c>
+      <c r="O6">
+        <v>9.9</v>
+      </c>
+      <c r="P6">
+        <v>-9.9</v>
+      </c>
+      <c r="Q6">
+        <v>3</v>
+      </c>
+      <c r="R6">
+        <v>0.03</v>
+      </c>
+      <c r="S6">
+        <v>4</v>
+      </c>
+      <c r="T6">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>231</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>231</v>
+      </c>
+      <c r="E7" t="s">
+        <v>173</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0.02</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0.47099999999999997</v>
+      </c>
+      <c r="K7">
+        <v>1.3</v>
+      </c>
+      <c r="L7">
+        <v>0.23</v>
+      </c>
+      <c r="M7">
+        <v>10.1</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <v>5</v>
+      </c>
+      <c r="P7">
+        <v>-5</v>
+      </c>
+      <c r="Q7">
+        <v>3</v>
+      </c>
+      <c r="R7">
+        <v>0.08</v>
+      </c>
+      <c r="S7">
+        <v>4</v>
+      </c>
+      <c r="T7">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>232</v>
+      </c>
+      <c r="E8" t="s">
+        <v>174</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0.02</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0.73</v>
+      </c>
+      <c r="K8">
+        <v>1.3</v>
+      </c>
+      <c r="L8">
+        <v>0.23</v>
+      </c>
+      <c r="M8">
+        <v>40</v>
+      </c>
+      <c r="N8">
+        <v>1</v>
+      </c>
+      <c r="O8">
+        <v>6.5</v>
+      </c>
+      <c r="P8">
+        <v>-6.5</v>
+      </c>
+      <c r="Q8">
+        <v>3</v>
+      </c>
+      <c r="R8">
+        <v>0.03</v>
+      </c>
+      <c r="S8">
+        <v>4</v>
+      </c>
+      <c r="T8">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E9" t="s">
+        <v>175</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0.02</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0.52800000000000002</v>
+      </c>
+      <c r="K9">
+        <v>1.3</v>
+      </c>
+      <c r="L9">
+        <v>0.23</v>
+      </c>
+      <c r="M9">
+        <v>10.1</v>
+      </c>
+      <c r="N9">
+        <v>-0.05</v>
+      </c>
+      <c r="O9">
+        <v>5</v>
+      </c>
+      <c r="P9">
+        <v>-5</v>
+      </c>
+      <c r="Q9">
+        <v>3</v>
+      </c>
+      <c r="R9">
+        <v>0.09</v>
+      </c>
+      <c r="S9">
+        <v>4</v>
+      </c>
+      <c r="T9">
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>234</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>234</v>
+      </c>
+      <c r="E10" t="s">
+        <v>176</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0.02</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0.95</v>
+      </c>
+      <c r="K10">
+        <v>1.3</v>
+      </c>
+      <c r="L10">
+        <v>0.23</v>
+      </c>
+      <c r="M10">
+        <v>40</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10">
+        <v>9.9</v>
+      </c>
+      <c r="P10">
+        <v>-9.9</v>
+      </c>
+      <c r="Q10">
+        <v>3</v>
+      </c>
+      <c r="R10">
+        <v>0.03</v>
+      </c>
+      <c r="S10">
+        <v>4</v>
+      </c>
+      <c r="T10">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>235</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>235</v>
+      </c>
+      <c r="E11" t="s">
+        <v>177</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0.02</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0.95</v>
+      </c>
+      <c r="K11">
+        <v>1.3</v>
+      </c>
+      <c r="L11">
+        <v>0.23</v>
+      </c>
+      <c r="M11">
+        <v>10.1</v>
+      </c>
+      <c r="N11">
+        <v>1</v>
+      </c>
+      <c r="O11">
+        <v>9.9</v>
+      </c>
+      <c r="P11">
+        <v>-9.9</v>
+      </c>
+      <c r="Q11">
+        <v>3</v>
+      </c>
+      <c r="R11">
+        <v>0.03</v>
+      </c>
+      <c r="S11">
+        <v>4</v>
+      </c>
+      <c r="T11">
+        <v>0.85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3357,7 +5034,7 @@
         <v>0.02</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -3383,7 +5060,7 @@
         <v>0.02</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -3409,7 +5086,7 @@
         <v>0.02</v>
       </c>
       <c r="H4">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -3435,7 +5112,7 @@
         <v>0.02</v>
       </c>
       <c r="H5">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -3461,7 +5138,7 @@
         <v>0.02</v>
       </c>
       <c r="H6">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -3487,7 +5164,7 @@
         <v>0.02</v>
       </c>
       <c r="H7">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -3513,7 +5190,7 @@
         <v>0.02</v>
       </c>
       <c r="H8">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -3539,7 +5216,7 @@
         <v>0.02</v>
       </c>
       <c r="H9">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -3565,7 +5242,7 @@
         <v>0.02</v>
       </c>
       <c r="H10">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -3591,7 +5268,7 @@
         <v>0.02</v>
       </c>
       <c r="H11">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -4425,7 +6102,7 @@
         <v>1.4</v>
       </c>
       <c r="Q2" s="6">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R2" s="6">
         <v>1.4E-3</v>
@@ -4481,7 +6158,7 @@
         <v>1.4</v>
       </c>
       <c r="Q3">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R3">
         <v>2.7E-2</v>
@@ -4537,7 +6214,7 @@
         <v>1.4</v>
       </c>
       <c r="Q4">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R4">
         <v>3.8600000000000001E-3</v>
@@ -4593,7 +6270,7 @@
         <v>1.4</v>
       </c>
       <c r="Q5">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R5">
         <v>2.2200000000000002E-3</v>
@@ -4649,7 +6326,7 @@
         <v>1.4</v>
       </c>
       <c r="Q6">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R6">
         <v>1.4E-3</v>
@@ -4706,7 +6383,7 @@
         <v>1.4</v>
       </c>
       <c r="Q7" s="6">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R7" s="6">
         <v>6.1499999999999999E-2</v>
@@ -4762,7 +6439,7 @@
         <v>1.4</v>
       </c>
       <c r="Q8">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R8">
         <v>2.6800000000000001E-3</v>
@@ -4819,7 +6496,7 @@
         <v>1.4</v>
       </c>
       <c r="Q9" s="6">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R9" s="6">
         <v>6.8599999999999998E-3</v>
@@ -4876,7 +6553,7 @@
         <v>1.4</v>
       </c>
       <c r="Q10" s="6">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R10" s="6">
         <v>3.0000000000000001E-3</v>
@@ -5148,7 +6825,7 @@
         <v>1</v>
       </c>
       <c r="J2">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -5180,7 +6857,7 @@
         <v>2</v>
       </c>
       <c r="J3">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -5287,10 +6964,10 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I2">
         <v>345</v>
@@ -5352,10 +7029,10 @@
         <v>39</v>
       </c>
       <c r="G3">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I3">
         <v>345</v>
@@ -5417,10 +7094,10 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="H4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I4">
         <v>345</v>
@@ -5482,10 +7159,10 @@
         <v>25</v>
       </c>
       <c r="G5">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="H5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I5">
         <v>345</v>
@@ -5547,10 +7224,10 @@
         <v>4</v>
       </c>
       <c r="G6">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H6">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I6">
         <v>345</v>
@@ -5612,10 +7289,10 @@
         <v>18</v>
       </c>
       <c r="G7">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="H7">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I7">
         <v>345</v>
@@ -5677,10 +7354,10 @@
         <v>5</v>
       </c>
       <c r="G8">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="H8">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I8">
         <v>345</v>
@@ -5742,10 +7419,10 @@
         <v>14</v>
       </c>
       <c r="G9">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H9">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I9">
         <v>345</v>
@@ -5807,10 +7484,10 @@
         <v>6</v>
       </c>
       <c r="G10">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="H10">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I10">
         <v>345</v>
@@ -5872,10 +7549,10 @@
         <v>8</v>
       </c>
       <c r="G11">
-        <v>100</v>
+        <v>1200</v>
       </c>
       <c r="H11">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I11">
         <v>345</v>
@@ -5937,10 +7614,10 @@
         <v>7</v>
       </c>
       <c r="G12">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H12">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I12">
         <v>345</v>
@@ -6002,10 +7679,10 @@
         <v>11</v>
       </c>
       <c r="G13">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H13">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I13">
         <v>345</v>
@@ -6067,10 +7744,10 @@
         <v>8</v>
       </c>
       <c r="G14">
-        <v>100</v>
+        <v>480</v>
       </c>
       <c r="H14">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I14">
         <v>345</v>
@@ -6132,10 +7809,10 @@
         <v>9</v>
       </c>
       <c r="G15">
-        <v>100</v>
+        <v>1800</v>
       </c>
       <c r="H15">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I15">
         <v>345</v>
@@ -6197,10 +7874,10 @@
         <v>39</v>
       </c>
       <c r="G16">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H16">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I16">
         <v>345</v>
@@ -6262,10 +7939,10 @@
         <v>11</v>
       </c>
       <c r="G17">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H17">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I17">
         <v>345</v>
@@ -6327,10 +8004,10 @@
         <v>13</v>
       </c>
       <c r="G18">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H18">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I18">
         <v>345</v>
@@ -6392,10 +8069,10 @@
         <v>14</v>
       </c>
       <c r="G19">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H19">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I19">
         <v>345</v>
@@ -6457,10 +8134,10 @@
         <v>15</v>
       </c>
       <c r="G20">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H20">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I20">
         <v>345</v>
@@ -6522,10 +8199,10 @@
         <v>16</v>
       </c>
       <c r="G21">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H21">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I21">
         <v>345</v>
@@ -6587,10 +8264,10 @@
         <v>17</v>
       </c>
       <c r="G22">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="H22">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I22">
         <v>345</v>
@@ -6651,11 +8328,11 @@
       <c r="F23">
         <v>19</v>
       </c>
-      <c r="G23">
-        <v>100</v>
+      <c r="G23" s="6">
+        <v>500</v>
       </c>
       <c r="H23">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I23">
         <v>345</v>
@@ -6717,10 +8394,10 @@
         <v>21</v>
       </c>
       <c r="G24">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H24">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I24">
         <v>345</v>
@@ -6782,10 +8459,10 @@
         <v>24</v>
       </c>
       <c r="G25">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H25">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I25">
         <v>345</v>
@@ -6847,10 +8524,10 @@
         <v>18</v>
       </c>
       <c r="G26">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H26">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I26">
         <v>345</v>
@@ -6912,10 +8589,10 @@
         <v>27</v>
       </c>
       <c r="G27">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H27">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I27">
         <v>345</v>
@@ -6977,10 +8654,10 @@
         <v>22</v>
       </c>
       <c r="G28">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H28">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I28">
         <v>345</v>
@@ -7042,10 +8719,10 @@
         <v>23</v>
       </c>
       <c r="G29">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H29">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I29">
         <v>345</v>
@@ -7107,10 +8784,10 @@
         <v>24</v>
       </c>
       <c r="G30">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H30">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I30">
         <v>345</v>
@@ -7172,10 +8849,10 @@
         <v>26</v>
       </c>
       <c r="G31">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H31">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I31">
         <v>345</v>
@@ -7237,10 +8914,10 @@
         <v>27</v>
       </c>
       <c r="G32">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H32">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I32">
         <v>345</v>
@@ -7302,10 +8979,10 @@
         <v>28</v>
       </c>
       <c r="G33">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H33">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I33">
         <v>345</v>
@@ -7367,10 +9044,10 @@
         <v>29</v>
       </c>
       <c r="G34">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H34">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I34">
         <v>345</v>
@@ -7432,10 +9109,10 @@
         <v>29</v>
       </c>
       <c r="G35">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H35">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I35">
         <v>345</v>
@@ -7496,11 +9173,11 @@
       <c r="F36">
         <v>30</v>
       </c>
-      <c r="G36">
-        <v>100</v>
+      <c r="G36" s="6">
+        <v>900</v>
       </c>
       <c r="H36">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I36">
         <v>345</v>
@@ -7561,11 +9238,11 @@
       <c r="F37">
         <v>6</v>
       </c>
-      <c r="G37">
-        <v>100</v>
+      <c r="G37" s="6">
+        <v>600</v>
       </c>
       <c r="H37">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I37">
         <v>34.5</v>
@@ -7626,11 +9303,11 @@
       <c r="F38">
         <v>32</v>
       </c>
-      <c r="G38">
-        <v>100</v>
+      <c r="G38" s="6">
+        <v>900</v>
       </c>
       <c r="H38">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I38">
         <v>345</v>
@@ -7692,10 +9369,10 @@
         <v>11</v>
       </c>
       <c r="G39">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H39">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I39">
         <v>138</v>
@@ -7757,10 +9434,10 @@
         <v>13</v>
       </c>
       <c r="G40">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H40">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I40">
         <v>138</v>
@@ -7821,11 +9498,11 @@
       <c r="F41">
         <v>20</v>
       </c>
-      <c r="G41">
-        <v>100</v>
+      <c r="G41" s="6">
+        <v>600</v>
       </c>
       <c r="H41">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I41">
         <v>345</v>
@@ -7886,11 +9563,11 @@
       <c r="F42">
         <v>33</v>
       </c>
-      <c r="G42">
-        <v>100</v>
+      <c r="G42" s="6">
+        <v>900</v>
       </c>
       <c r="H42">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I42">
         <v>345</v>
@@ -7951,11 +9628,11 @@
       <c r="F43">
         <v>34</v>
       </c>
-      <c r="G43">
-        <v>100</v>
+      <c r="G43" s="6">
+        <v>600</v>
       </c>
       <c r="H43">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I43">
         <v>138</v>
@@ -8016,11 +9693,11 @@
       <c r="F44">
         <v>35</v>
       </c>
-      <c r="G44">
-        <v>100</v>
+      <c r="G44" s="6">
+        <v>600</v>
       </c>
       <c r="H44">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I44">
         <v>345</v>
@@ -8081,11 +9758,11 @@
       <c r="F45">
         <v>36</v>
       </c>
-      <c r="G45">
-        <v>100</v>
+      <c r="G45" s="6">
+        <v>600</v>
       </c>
       <c r="H45">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I45">
         <v>345</v>
@@ -8146,11 +9823,11 @@
       <c r="F46">
         <v>37</v>
       </c>
-      <c r="G46">
-        <v>100</v>
+      <c r="G46" s="6">
+        <v>600</v>
       </c>
       <c r="H46">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I46">
         <v>345</v>
@@ -8211,11 +9888,11 @@
       <c r="F47">
         <v>38</v>
       </c>
-      <c r="G47">
-        <v>100</v>
+      <c r="G47" s="6">
+        <v>1200</v>
       </c>
       <c r="H47">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I47">
         <v>345</v>
@@ -8427,6 +10104,9 @@
       <c r="F2">
         <v>1</v>
       </c>
+      <c r="G2" t="s">
+        <v>210</v>
+      </c>
       <c r="H2">
         <v>1040</v>
       </c>
@@ -8434,7 +10114,7 @@
         <v>34.5</v>
       </c>
       <c r="J2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -8520,7 +10200,7 @@
         <v>34.5</v>
       </c>
       <c r="J3">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -8606,7 +10286,7 @@
         <v>21</v>
       </c>
       <c r="J4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -8692,7 +10372,7 @@
         <v>21</v>
       </c>
       <c r="J5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -8778,7 +10458,7 @@
         <v>15.5</v>
       </c>
       <c r="J6">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -8854,6 +10534,9 @@
       <c r="F7">
         <v>6</v>
       </c>
+      <c r="G7" t="s">
+        <v>210</v>
+      </c>
       <c r="H7">
         <v>1085.7</v>
       </c>
@@ -8861,7 +10544,7 @@
         <v>15.5</v>
       </c>
       <c r="J7">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -8947,7 +10630,7 @@
         <v>12.5</v>
       </c>
       <c r="J8">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -9023,6 +10706,9 @@
       <c r="F9">
         <v>8</v>
       </c>
+      <c r="G9" t="s">
+        <v>210</v>
+      </c>
       <c r="H9">
         <v>970.2</v>
       </c>
@@ -9030,7 +10716,7 @@
         <v>12.5</v>
       </c>
       <c r="J9">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -9106,6 +10792,9 @@
       <c r="F10">
         <v>9</v>
       </c>
+      <c r="G10" t="s">
+        <v>210</v>
+      </c>
       <c r="H10">
         <v>1684.1</v>
       </c>
@@ -9113,7 +10802,7 @@
         <v>34.5</v>
       </c>
       <c r="J10">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -9199,13 +10888,13 @@
         <v>345</v>
       </c>
       <c r="J11">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="M11">
         <v>1E-3</v>

</xml_diff>